<commit_message>
se agrega dos carpetas de proyecto el modelo 3 que se tarbaja por keywordtest estilo combinacion screenplay y POM se agrega el escenario de login logout completo
</commit_message>
<xml_diff>
--- a/Banca en Linea modelo 1/Datos/Datos.xlsx
+++ b/Banca en Linea modelo 1/Datos/Datos.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bespinosa\Documents\Katalon\Demo Banca en Linea\Demo-Banca-en-Linea\Banca en Linea modelo 1\Datos\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44478314-62A0-48EF-92A7-6E99D799ADFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,52 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>gcambiso15</t>
+  </si>
+  <si>
+    <t>Ftolb123</t>
+  </si>
+  <si>
+    <t>prueba</t>
+  </si>
+  <si>
+    <t>jose@gmail.com</t>
+  </si>
+  <si>
+    <t>2344235353423</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>cuenta</t>
+  </si>
+  <si>
+    <t>monto</t>
+  </si>
+  <si>
+    <t>concepto</t>
+  </si>
+  <si>
+    <t>correo</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>http://10.10.23.211:8280/mcm-web-render/pages/index.jsp</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,8 +99,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +392,119 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" customWidth="1"/>
+    <col min="3" max="4" width="18.81640625" customWidth="1"/>
+    <col min="5" max="5" width="22.08984375" customWidth="1"/>
+    <col min="6" max="6" width="24.81640625" customWidth="1"/>
+    <col min="7" max="7" width="46.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{289b8e9f-7030-4088-924a-9be7e27c9057}" enabled="1" method="Standard" siteId="{d452ab8e-715a-472d-8c25-66f6a48ce997}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>